<commit_message>
Add 8 more Aizu stations resolved from user follow-up (28 total)
Adds 湯川橋, 鶴沼橋, 馬越, 小豆沢, 一の戸川, 宮川, 大谷川, 大橋 to cameras.csv
(coordinates from river.go.jp per-station pages, same workflow as the initial
20-station Aizu batch) and extends the Aizu xlsx header template's station
columns to match. 大石 and 宮古 were investigated but have no photo camera on
river.go.jp under those names (only water-level gauges), so they're excluded.
</commit_message>
<xml_diff>
--- a/template/header_template_aizu.xlsx
+++ b/template/header_template_aizu.xlsx
@@ -1281,14 +1281,46 @@
           <t>南大橋</t>
         </is>
       </c>
-      <c r="AW1" s="3" t="n"/>
-      <c r="AX1" s="3" t="n"/>
-      <c r="AY1" s="3" t="n"/>
-      <c r="AZ1" s="3" t="n"/>
-      <c r="BA1" s="3" t="n"/>
-      <c r="BB1" s="3" t="n"/>
-      <c r="BC1" s="3" t="n"/>
-      <c r="BD1" s="3" t="n"/>
+      <c r="AW1" s="3" t="inlineStr">
+        <is>
+          <t>湯川橋</t>
+        </is>
+      </c>
+      <c r="AX1" s="3" t="inlineStr">
+        <is>
+          <t>鶴沼橋</t>
+        </is>
+      </c>
+      <c r="AY1" s="3" t="inlineStr">
+        <is>
+          <t>馬越</t>
+        </is>
+      </c>
+      <c r="AZ1" s="3" t="inlineStr">
+        <is>
+          <t>小豆沢</t>
+        </is>
+      </c>
+      <c r="BA1" s="3" t="inlineStr">
+        <is>
+          <t>一の戸川</t>
+        </is>
+      </c>
+      <c r="BB1" s="3" t="inlineStr">
+        <is>
+          <t>宮川</t>
+        </is>
+      </c>
+      <c r="BC1" s="3" t="inlineStr">
+        <is>
+          <t>大谷川</t>
+        </is>
+      </c>
+      <c r="BD1" s="3" t="inlineStr">
+        <is>
+          <t>大橋</t>
+        </is>
+      </c>
       <c r="BE1" s="3" t="n"/>
       <c r="BF1" s="3" t="n"/>
       <c r="BG1" s="2" t="n"/>

</xml_diff>

<commit_message>
Add the last requested Aizu station (大石)
The originally requested 32-point Aizu list is now complete. The
station shares its name with an unrelated 危機管理型水位計 (simple
water-level gauge, itmkndCd=300) with no camera at all, which is why
earlier keyword searches kept surfacing that one instead; the real
camera entry (itmkndCd=200, camera id 121527029) has a working live
image and was found via the direct station URL.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JKyDPYhW8rAcdQCbd9XRYd
</commit_message>
<xml_diff>
--- a/template/header_template_aizu.xlsx
+++ b/template/header_template_aizu.xlsx
@@ -1336,7 +1336,11 @@
           <t>福島</t>
         </is>
       </c>
-      <c r="BH1" s="3" t="n"/>
+      <c r="BH1" s="3" t="inlineStr">
+        <is>
+          <t>大石</t>
+        </is>
+      </c>
       <c r="BI1" s="3" t="n"/>
     </row>
     <row r="2">

</xml_diff>